<commit_message>
Update Render Disk Fix
</commit_message>
<xml_diff>
--- a/position_cleanup_results.xlsx
+++ b/position_cleanup_results.xlsx
@@ -8,9 +8,9 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="https://d.docs.live.net/cb4a1c0c7a4389a8/Documents/GitHub/GoLive_Staffing/"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="8" documentId="11_6F29C2F7EBF38B6B0F6440E6A16F09F978795FE3" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{096BF7CA-CC30-4792-9A76-9FEEAC901433}"/>
+  <xr:revisionPtr revIDLastSave="10" documentId="11_6F29C2F7EBF38B6B0F6440E6A16F09F978795FE3" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{59C3F2C7-CDF4-4C56-9878-E71BD26180B5}"/>
   <bookViews>
-    <workbookView xWindow="28680" yWindow="-120" windowWidth="29040" windowHeight="15720" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
+    <workbookView xWindow="28680" yWindow="-4560" windowWidth="38640" windowHeight="21120" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
   <sheets>
     <sheet name="Sheet1" sheetId="1" r:id="rId1"/>
@@ -655,7 +655,7 @@
       <scheme val="minor"/>
     </font>
   </fonts>
-  <fills count="3">
+  <fills count="4">
     <fill>
       <patternFill patternType="none"/>
     </fill>
@@ -665,6 +665,12 @@
     <fill>
       <patternFill patternType="solid">
         <fgColor rgb="FFFFFF00"/>
+        <bgColor indexed="64"/>
+      </patternFill>
+    </fill>
+    <fill>
+      <patternFill patternType="solid">
+        <fgColor theme="6" tint="0.59999389629810485"/>
         <bgColor indexed="64"/>
       </patternFill>
     </fill>
@@ -696,7 +702,7 @@
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="5">
+  <cellXfs count="7">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
     <xf numFmtId="0" fontId="1" fillId="0" borderId="1" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="top"/>
@@ -706,6 +712,10 @@
       <alignment horizontal="center" vertical="top"/>
     </xf>
     <xf numFmtId="0" fontId="0" fillId="2" borderId="0" xfId="0" applyFill="1"/>
+    <xf numFmtId="0" fontId="1" fillId="3" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="top"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="3" borderId="0" xfId="0" applyFill="1"/>
   </cellXfs>
   <cellStyles count="1">
     <cellStyle name="Normal" xfId="0" builtinId="0"/>
@@ -1018,7 +1028,8 @@
     <col min="3" max="3" width="9.42578125" bestFit="1" customWidth="1"/>
     <col min="4" max="4" width="17.42578125" bestFit="1" customWidth="1"/>
     <col min="5" max="5" width="13.7109375" bestFit="1" customWidth="1"/>
-    <col min="6" max="7" width="20.7109375" customWidth="1"/>
+    <col min="6" max="6" width="20.7109375" customWidth="1"/>
+    <col min="7" max="7" width="100.140625" customWidth="1"/>
     <col min="8" max="8" width="70.140625" style="4" bestFit="1" customWidth="1"/>
     <col min="9" max="9" width="13.5703125" bestFit="1" customWidth="1"/>
   </cols>
@@ -1033,7 +1044,7 @@
       <c r="C1" s="1" t="s">
         <v>2</v>
       </c>
-      <c r="D1" s="1" t="s">
+      <c r="D1" s="5" t="s">
         <v>3</v>
       </c>
       <c r="E1" s="1" t="s">
@@ -1062,7 +1073,7 @@
       <c r="C2">
         <v>112183</v>
       </c>
-      <c r="D2" t="s">
+      <c r="D2" s="6" t="s">
         <v>14</v>
       </c>
       <c r="E2" t="s">
@@ -1091,7 +1102,7 @@
       <c r="C3">
         <v>111906</v>
       </c>
-      <c r="D3" t="s">
+      <c r="D3" s="6" t="s">
         <v>18</v>
       </c>
       <c r="E3" t="s">
@@ -1120,7 +1131,7 @@
       <c r="C4">
         <v>112130</v>
       </c>
-      <c r="D4" t="s">
+      <c r="D4" s="6" t="s">
         <v>21</v>
       </c>
       <c r="E4" t="s">
@@ -1149,7 +1160,7 @@
       <c r="C5">
         <v>112155</v>
       </c>
-      <c r="D5" t="s">
+      <c r="D5" s="6" t="s">
         <v>23</v>
       </c>
       <c r="E5" t="s">
@@ -1178,7 +1189,7 @@
       <c r="C6">
         <v>112160</v>
       </c>
-      <c r="D6" t="s">
+      <c r="D6" s="6" t="s">
         <v>24</v>
       </c>
       <c r="E6" t="s">
@@ -1207,7 +1218,7 @@
       <c r="C7">
         <v>112160</v>
       </c>
-      <c r="D7" t="s">
+      <c r="D7" s="6" t="s">
         <v>24</v>
       </c>
       <c r="E7" t="s">
@@ -1236,7 +1247,7 @@
       <c r="C8">
         <v>104265</v>
       </c>
-      <c r="D8" t="s">
+      <c r="D8" s="6" t="s">
         <v>26</v>
       </c>
       <c r="E8" t="s">
@@ -1265,7 +1276,7 @@
       <c r="C9">
         <v>9631</v>
       </c>
-      <c r="D9" t="s">
+      <c r="D9" s="6" t="s">
         <v>32</v>
       </c>
       <c r="E9" t="s">
@@ -1294,7 +1305,7 @@
       <c r="C10">
         <v>15756</v>
       </c>
-      <c r="D10" t="s">
+      <c r="D10" s="6" t="s">
         <v>35</v>
       </c>
       <c r="E10" t="s">
@@ -1323,7 +1334,7 @@
       <c r="C11">
         <v>111558</v>
       </c>
-      <c r="D11" t="s">
+      <c r="D11" s="6" t="s">
         <v>38</v>
       </c>
       <c r="E11" t="s">
@@ -1352,7 +1363,7 @@
       <c r="C12">
         <v>112102</v>
       </c>
-      <c r="D12" t="s">
+      <c r="D12" s="6" t="s">
         <v>22</v>
       </c>
       <c r="E12" t="s">
@@ -1381,7 +1392,7 @@
       <c r="C13">
         <v>15756</v>
       </c>
-      <c r="D13" t="s">
+      <c r="D13" s="6" t="s">
         <v>35</v>
       </c>
       <c r="E13" t="s">
@@ -1410,7 +1421,7 @@
       <c r="C14">
         <v>110408</v>
       </c>
-      <c r="D14" t="s">
+      <c r="D14" s="6" t="s">
         <v>45</v>
       </c>
       <c r="E14" t="s">
@@ -1439,7 +1450,7 @@
       <c r="C15">
         <v>9631</v>
       </c>
-      <c r="D15" t="s">
+      <c r="D15" s="6" t="s">
         <v>32</v>
       </c>
       <c r="E15" t="s">
@@ -1468,7 +1479,7 @@
       <c r="C16">
         <v>101042</v>
       </c>
-      <c r="D16" t="s">
+      <c r="D16" s="6" t="s">
         <v>12</v>
       </c>
       <c r="E16" t="s">
@@ -1497,7 +1508,7 @@
       <c r="C17">
         <v>112180</v>
       </c>
-      <c r="D17" t="s">
+      <c r="D17" s="6" t="s">
         <v>13</v>
       </c>
       <c r="E17" t="s">
@@ -1526,7 +1537,7 @@
       <c r="C18">
         <v>112180</v>
       </c>
-      <c r="D18" t="s">
+      <c r="D18" s="6" t="s">
         <v>13</v>
       </c>
       <c r="E18" t="s">
@@ -1555,7 +1566,7 @@
       <c r="C19">
         <v>112273</v>
       </c>
-      <c r="D19" t="s">
+      <c r="D19" s="6" t="s">
         <v>16</v>
       </c>
       <c r="E19" t="s">
@@ -1584,7 +1595,7 @@
       <c r="C20">
         <v>111927</v>
       </c>
-      <c r="D20" t="s">
+      <c r="D20" s="6" t="s">
         <v>17</v>
       </c>
       <c r="E20" t="s">
@@ -1613,7 +1624,7 @@
       <c r="C21">
         <v>112082</v>
       </c>
-      <c r="D21" t="s">
+      <c r="D21" s="6" t="s">
         <v>19</v>
       </c>
       <c r="E21" t="s">
@@ -1642,7 +1653,7 @@
       <c r="C22">
         <v>112170</v>
       </c>
-      <c r="D22" t="s">
+      <c r="D22" s="6" t="s">
         <v>20</v>
       </c>
       <c r="E22" t="s">
@@ -1671,7 +1682,7 @@
       <c r="C23">
         <v>112082</v>
       </c>
-      <c r="D23" t="s">
+      <c r="D23" s="6" t="s">
         <v>19</v>
       </c>
       <c r="E23" t="s">
@@ -1700,7 +1711,7 @@
       <c r="C24">
         <v>112102</v>
       </c>
-      <c r="D24" t="s">
+      <c r="D24" s="6" t="s">
         <v>22</v>
       </c>
       <c r="E24" t="s">
@@ -1729,7 +1740,7 @@
       <c r="C25">
         <v>110124</v>
       </c>
-      <c r="D25" t="s">
+      <c r="D25" s="6" t="s">
         <v>25</v>
       </c>
       <c r="E25" t="s">
@@ -1758,7 +1769,7 @@
       <c r="C26">
         <v>110124</v>
       </c>
-      <c r="D26" t="s">
+      <c r="D26" s="6" t="s">
         <v>25</v>
       </c>
       <c r="E26" t="s">
@@ -1787,7 +1798,7 @@
       <c r="C27">
         <v>112107</v>
       </c>
-      <c r="D27" t="s">
+      <c r="D27" s="6" t="s">
         <v>30</v>
       </c>
       <c r="E27" t="s">
@@ -1816,7 +1827,7 @@
       <c r="C28">
         <v>110959</v>
       </c>
-      <c r="D28" t="s">
+      <c r="D28" s="6" t="s">
         <v>31</v>
       </c>
       <c r="E28" t="s">
@@ -1845,7 +1856,7 @@
       <c r="C29">
         <v>112107</v>
       </c>
-      <c r="D29" t="s">
+      <c r="D29" s="6" t="s">
         <v>30</v>
       </c>
       <c r="E29" t="s">
@@ -1874,7 +1885,7 @@
       <c r="C30">
         <v>103543</v>
       </c>
-      <c r="D30" t="s">
+      <c r="D30" s="6" t="s">
         <v>33</v>
       </c>
       <c r="E30" t="s">
@@ -1903,7 +1914,7 @@
       <c r="C31">
         <v>112102</v>
       </c>
-      <c r="D31" t="s">
+      <c r="D31" s="6" t="s">
         <v>22</v>
       </c>
       <c r="E31" t="s">
@@ -1932,7 +1943,7 @@
       <c r="C32">
         <v>112120</v>
       </c>
-      <c r="D32" t="s">
+      <c r="D32" s="6" t="s">
         <v>36</v>
       </c>
       <c r="E32" t="s">
@@ -1961,7 +1972,7 @@
       <c r="C33">
         <v>112167</v>
       </c>
-      <c r="D33" t="s">
+      <c r="D33" s="6" t="s">
         <v>39</v>
       </c>
       <c r="E33" t="s">
@@ -1990,7 +2001,7 @@
       <c r="C34">
         <v>103543</v>
       </c>
-      <c r="D34" t="s">
+      <c r="D34" s="6" t="s">
         <v>33</v>
       </c>
       <c r="E34" t="s">
@@ -2019,7 +2030,7 @@
       <c r="C35">
         <v>111677</v>
       </c>
-      <c r="D35" t="s">
+      <c r="D35" s="6" t="s">
         <v>42</v>
       </c>
       <c r="E35" t="s">
@@ -2048,7 +2059,7 @@
       <c r="C36">
         <v>108990</v>
       </c>
-      <c r="D36" t="s">
+      <c r="D36" s="6" t="s">
         <v>43</v>
       </c>
       <c r="E36" t="s">
@@ -2077,7 +2088,7 @@
       <c r="C37">
         <v>112112</v>
       </c>
-      <c r="D37" t="s">
+      <c r="D37" s="6" t="s">
         <v>44</v>
       </c>
       <c r="E37" t="s">
@@ -2106,7 +2117,7 @@
       <c r="C38">
         <v>112069</v>
       </c>
-      <c r="D38" t="s">
+      <c r="D38" s="6" t="s">
         <v>46</v>
       </c>
       <c r="E38" t="s">
@@ -2135,7 +2146,7 @@
       <c r="C39">
         <v>108227</v>
       </c>
-      <c r="D39" t="s">
+      <c r="D39" s="6" t="s">
         <v>47</v>
       </c>
       <c r="E39" t="s">
@@ -2164,7 +2175,7 @@
       <c r="C40">
         <v>102244</v>
       </c>
-      <c r="D40" t="s">
+      <c r="D40" s="6" t="s">
         <v>48</v>
       </c>
       <c r="E40" t="s">
@@ -2193,7 +2204,7 @@
       <c r="C41">
         <v>18885</v>
       </c>
-      <c r="D41" t="s">
+      <c r="D41" s="6" t="s">
         <v>49</v>
       </c>
       <c r="E41" t="s">
@@ -2222,7 +2233,7 @@
       <c r="C42">
         <v>112176</v>
       </c>
-      <c r="D42" t="s">
+      <c r="D42" s="6" t="s">
         <v>15</v>
       </c>
       <c r="E42" t="s">
@@ -2248,7 +2259,7 @@
       <c r="C43">
         <v>112160</v>
       </c>
-      <c r="D43" t="s">
+      <c r="D43" s="6" t="s">
         <v>24</v>
       </c>
       <c r="E43" t="s">
@@ -2274,7 +2285,7 @@
       <c r="C44">
         <v>111875</v>
       </c>
-      <c r="D44" t="s">
+      <c r="D44" s="6" t="s">
         <v>27</v>
       </c>
       <c r="E44" t="s">
@@ -2300,7 +2311,7 @@
       <c r="C45">
         <v>112155</v>
       </c>
-      <c r="D45" t="s">
+      <c r="D45" s="6" t="s">
         <v>23</v>
       </c>
       <c r="E45" t="s">
@@ -2326,7 +2337,7 @@
       <c r="C46">
         <v>108381</v>
       </c>
-      <c r="D46" t="s">
+      <c r="D46" s="6" t="s">
         <v>28</v>
       </c>
       <c r="E46" t="s">
@@ -2352,7 +2363,7 @@
       <c r="C47">
         <v>110330</v>
       </c>
-      <c r="D47" t="s">
+      <c r="D47" s="6" t="s">
         <v>29</v>
       </c>
       <c r="E47" t="s">
@@ -2378,7 +2389,7 @@
       <c r="C48">
         <v>112102</v>
       </c>
-      <c r="D48" t="s">
+      <c r="D48" s="6" t="s">
         <v>22</v>
       </c>
       <c r="E48" t="s">
@@ -2404,7 +2415,7 @@
       <c r="C49">
         <v>110151</v>
       </c>
-      <c r="D49" t="s">
+      <c r="D49" s="6" t="s">
         <v>34</v>
       </c>
       <c r="E49" t="s">
@@ -2430,7 +2441,7 @@
       <c r="C50">
         <v>102628</v>
       </c>
-      <c r="D50" t="s">
+      <c r="D50" s="6" t="s">
         <v>37</v>
       </c>
       <c r="E50" t="s">
@@ -2456,7 +2467,7 @@
       <c r="C51">
         <v>110365</v>
       </c>
-      <c r="D51" t="s">
+      <c r="D51" s="6" t="s">
         <v>40</v>
       </c>
       <c r="E51" t="s">
@@ -2482,7 +2493,7 @@
       <c r="C52">
         <v>112088</v>
       </c>
-      <c r="D52" t="s">
+      <c r="D52" s="6" t="s">
         <v>41</v>
       </c>
       <c r="E52" t="s">

</xml_diff>